<commit_message>
Track M3 source files and clean workbook formatting
</commit_message>
<xml_diff>
--- a/Academic_documents/resultados CIA y LASA muestreo 2/muestreo2_solidos_volatiles.xlsx
+++ b/Academic_documents/resultados CIA y LASA muestreo 2/muestreo2_solidos_volatiles.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mateo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mateo\Downloads\LCA_IPCC_MANURE_TURRIALBA_UCR\Academic_documents\resultados CIA y LASA muestreo 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D0A1E9-0C6D-4C95-8C7B-37D1BE14812F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0F1FF4-3431-4952-904E-2C2231C862A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="960" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Procedure" sheetId="1" r:id="rId1"/>
@@ -508,20 +508,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -990,11 +990,11 @@
       <c r="A10" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
       <c r="E10" s="3" t="s">
         <v>2</v>
       </c>
@@ -1017,11 +1017,11 @@
       <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="18">
         <v>1</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
       <c r="E11" s="2" t="s">
         <v>3</v>
       </c>
@@ -1030,11 +1030,11 @@
       <c r="A12" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="18">
         <v>1</v>
       </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
       <c r="E12" s="2" t="s">
         <v>5</v>
       </c>
@@ -1043,11 +1043,11 @@
       <c r="A13" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="18">
         <v>1</v>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
       <c r="E13" s="2" t="s">
         <v>7</v>
       </c>
@@ -1056,11 +1056,11 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="18">
         <v>2</v>
       </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
       <c r="E14" s="2" t="s">
         <v>8</v>
       </c>
@@ -1069,11 +1069,11 @@
       <c r="A15" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="18">
         <v>2</v>
       </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
       <c r="E15" s="2" t="s">
         <v>10</v>
       </c>
@@ -1082,11 +1082,11 @@
       <c r="A16" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="18">
         <v>2</v>
       </c>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
       <c r="E16" s="2" t="s">
         <v>12</v>
       </c>
@@ -1095,11 +1095,11 @@
       <c r="A17" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="18">
         <v>12</v>
       </c>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
       <c r="E17" s="2" t="s">
         <v>27</v>
       </c>
@@ -1108,11 +1108,11 @@
       <c r="A18" t="s">
         <v>25</v>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="18">
         <v>12</v>
       </c>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
       <c r="E18" s="2" t="s">
         <v>24</v>
       </c>
@@ -1256,19 +1256,19 @@
         <f>((F2-J2)/F2)*100</f>
         <v>-34.119720466252495</v>
       </c>
-      <c r="L2" s="18">
+      <c r="L2" s="21">
         <f>MEDIAN(H2,H3,H4)</f>
         <v>86.809204218600172</v>
       </c>
-      <c r="M2" s="18">
+      <c r="M2" s="21">
         <f>MEDIAN(I2,I3,I4)</f>
         <v>13.190795781399824</v>
       </c>
-      <c r="N2" s="18">
+      <c r="N2" s="21">
         <f>AVERAGE(L2,L5)</f>
         <v>86.978418404265895</v>
       </c>
-      <c r="O2" s="18">
+      <c r="O2" s="21">
         <f>AVERAGE(M2,M5)</f>
         <v>13.021581595734107</v>
       </c>
@@ -1309,10 +1309,10 @@
         <f t="shared" ref="K3:K16" si="4">((F3-J3)/F3)*100</f>
         <v>3.4749306893473033</v>
       </c>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
+      <c r="O3" s="22"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -1350,10 +1350,10 @@
         <f t="shared" si="4"/>
         <v>1.4208862683119567</v>
       </c>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1391,16 +1391,16 @@
         <f t="shared" si="4"/>
         <v>17.414669330309057</v>
       </c>
-      <c r="L5" s="18">
+      <c r="L5" s="21">
         <f t="shared" ref="L5" si="5">MEDIAN(H5,H6,H7)</f>
         <v>87.147632589931618</v>
       </c>
-      <c r="M5" s="18">
+      <c r="M5" s="21">
         <f>MEDIAN(I5,I6,I7)</f>
         <v>12.852367410068389</v>
       </c>
-      <c r="N5" s="19"/>
-      <c r="O5" s="19"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -1438,10 +1438,10 @@
         <f t="shared" si="4"/>
         <v>-6.0235163010108179</v>
       </c>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1479,10 +1479,10 @@
         <f t="shared" si="4"/>
         <v>3.1771365869472947</v>
       </c>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="19"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="22"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1643,19 +1643,19 @@
         <f t="shared" si="4"/>
         <v>0.58803056888875482</v>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="21">
         <f t="shared" ref="L11" si="11">MEDIAN(H11,H12,H13)</f>
         <v>80.678915549769712</v>
       </c>
-      <c r="M11" s="18">
+      <c r="M11" s="21">
         <f>MEDIAN(I11,I12,I13)</f>
         <v>19.321084450230281</v>
       </c>
-      <c r="N11" s="18">
+      <c r="N11" s="21">
         <f>AVERAGE(L11,L14)</f>
         <v>81.221730305729992</v>
       </c>
-      <c r="O11" s="18">
+      <c r="O11" s="21">
         <f>AVERAGE(M11,M14)</f>
         <v>18.778269694270005</v>
       </c>
@@ -1696,10 +1696,10 @@
         <f t="shared" si="4"/>
         <v>-2.3503985196464976</v>
       </c>
-      <c r="L12" s="19"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19"/>
-      <c r="O12" s="19"/>
+      <c r="L12" s="22"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="22"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -1737,10 +1737,10 @@
         <f t="shared" si="4"/>
         <v>-22.365390053786314</v>
       </c>
-      <c r="L13" s="19"/>
-      <c r="M13" s="19"/>
-      <c r="N13" s="19"/>
-      <c r="O13" s="19"/>
+      <c r="L13" s="22"/>
+      <c r="M13" s="22"/>
+      <c r="N13" s="22"/>
+      <c r="O13" s="22"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1778,16 +1778,16 @@
         <f t="shared" si="4"/>
         <v>17.728573480504277</v>
       </c>
-      <c r="L14" s="18">
+      <c r="L14" s="21">
         <f t="shared" ref="L14" si="12">MEDIAN(H14,H15,H16)</f>
         <v>81.764545061690271</v>
       </c>
-      <c r="M14" s="18">
+      <c r="M14" s="21">
         <f>MEDIAN(I14,I15,I16)</f>
         <v>18.235454938309729</v>
       </c>
-      <c r="N14" s="19"/>
-      <c r="O14" s="19"/>
+      <c r="N14" s="22"/>
+      <c r="O14" s="22"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1825,10 +1825,10 @@
         <f t="shared" si="4"/>
         <v>0.47420766992036562</v>
       </c>
-      <c r="L15" s="19"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="19"/>
-      <c r="O15" s="19"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1866,10 +1866,10 @@
         <f t="shared" si="4"/>
         <v>18.022158372387125</v>
       </c>
-      <c r="L16" s="19"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
-      <c r="O16" s="19"/>
+      <c r="L16" s="22"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -2063,12 +2063,9 @@
         <f>(100-H22)</f>
         <v>82.484907207274347</v>
       </c>
-      <c r="J22">
-        <v>39.420200000000001</v>
-      </c>
       <c r="K22">
         <f>((F22-J22)/F22)*100</f>
-        <v>-11.87224719611315</v>
+        <v>100</v>
       </c>
       <c r="L22" s="20">
         <f>MEDIAN(H22,H23,H24)</f>
@@ -2947,14 +2944,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="O31:O36"/>
-    <mergeCell ref="L34:L36"/>
-    <mergeCell ref="M34:M36"/>
-    <mergeCell ref="M11:M13"/>
-    <mergeCell ref="M14:M16"/>
-    <mergeCell ref="L31:L33"/>
-    <mergeCell ref="M31:M33"/>
-    <mergeCell ref="N31:N36"/>
     <mergeCell ref="N2:N7"/>
     <mergeCell ref="O2:O7"/>
     <mergeCell ref="N11:N16"/>
@@ -2971,6 +2960,14 @@
     <mergeCell ref="L14:L16"/>
     <mergeCell ref="M2:M4"/>
     <mergeCell ref="M5:M7"/>
+    <mergeCell ref="O31:O36"/>
+    <mergeCell ref="L34:L36"/>
+    <mergeCell ref="M34:M36"/>
+    <mergeCell ref="M11:M13"/>
+    <mergeCell ref="M14:M16"/>
+    <mergeCell ref="L31:L33"/>
+    <mergeCell ref="M31:M33"/>
+    <mergeCell ref="N31:N36"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>